<commit_message>
navires par mois + adil + deploy scripts
</commit_message>
<xml_diff>
--- a/backend/security/users.xlsx
+++ b/backend/security/users.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,6 +535,32 @@
         </is>
       </c>
       <c r="F4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>adil.jiri</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AdiL1122</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Adil Jiri</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>analyst_2025_2026</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RBAC toutes années + fixes KPI marchandises/qualité
</commit_message>
<xml_diff>
--- a/backend/security/users.xlsx
+++ b/backend/security/users.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>analyst_2025_2026</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -501,7 +501,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>analyst_2026</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -554,10 +554,9 @@
           <t>Adil Jiri</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>analyst_2025_2026</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>